<commit_message>
a lot of changes to dave, he's slowly coming along, maybe it should be Infinite Dave and not infite RPG, fixes the problem about multiple classes B-), then i can finally focus on making the enemies work well
</commit_message>
<xml_diff>
--- a/ItemDataExcel.xlsx
+++ b/ItemDataExcel.xlsx
@@ -493,7 +493,7 @@
       </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>ItemSpeed</t>
+          <t>AttackSpeed</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
@@ -852,7 +852,7 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
@@ -965,7 +965,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t>Amulet</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -994,7 +994,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t>Ring</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t>Shoes</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1052,7 +1052,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t>Torso</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t>Helmet</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t>Pants</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1139,22 +1139,24 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>Offhand</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="C22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>Default</t>
-        </is>
-      </c>
       <c r="E22" t="n">
         <v>0</v>
       </c>
       <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>3</v>
+      </c>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
@@ -1168,24 +1170,28 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>Weapon</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="C23" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>Default</t>
-        </is>
-      </c>
       <c r="E23" t="n">
         <v>0</v>
       </c>
-      <c r="F23" t="inlineStr"/>
+      <c r="F23" t="n">
+        <v>5</v>
+      </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr"/>
+      <c r="I23" t="n">
+        <v>1.1</v>
+      </c>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
     </row>
@@ -1197,21 +1203,23 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
+          <t>Ring</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="C24" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>Default</t>
-        </is>
-      </c>
       <c r="E24" t="n">
         <v>0</v>
       </c>
-      <c r="F24" t="inlineStr"/>
+      <c r="F24" t="n">
+        <v>100</v>
+      </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
@@ -1226,21 +1234,23 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>Amulet</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
           <t>Default</t>
         </is>
       </c>
-      <c r="C25" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>Default</t>
-        </is>
-      </c>
       <c r="E25" t="n">
         <v>0</v>
       </c>
-      <c r="F25" t="inlineStr"/>
+      <c r="F25" t="n">
+        <v>100</v>
+      </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>

</xml_diff>

<commit_message>
made a lot of changes, added state machines for the enemies
</commit_message>
<xml_diff>
--- a/ItemDataExcel.xlsx
+++ b/ItemDataExcel.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://dtudk-my.sharepoint.com/personal/s225183_dtu_dk/Documents/ProjektGodot/Rapid RPG/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_7E1D701C952A91658113874AC8A9299979FB3072" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DDE0424F-0418-41F1-B668-95AE5979A807}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_7E1D701C952A91658113874AC8A9299979FB3072" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2E88057F-25FF-44F8-AA41-3AFF4F9A2651}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="3285" yWindow="1335" windowWidth="21510" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -574,6 +574,7 @@
   <dimension ref="A1:K29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="20.85546875" customWidth="1"/>
     <col min="2" max="2" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>